<commit_message>
Add Excel reading script and update workbook handling
Added leitura.py for reading and modifying Excel files using openpyxl. Updated main.py to create and access a new sheet named 'Teste', print sheet names, and append student data. Updated workbook.xlsx to reflect these changes. Also added a temporary file in the _csv directory.
</commit_message>
<xml_diff>
--- a/secao6/_openpyxl/workbook.xlsx
+++ b/secao6/_openpyxl/workbook.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Teste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,7 +486,72 @@
         <v>6.8</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ana Silva</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bruno Costa</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>18</v>
+      </c>
+      <c r="C7" t="n">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carla Mendes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Diego Rocha</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>17</v>
+      </c>
+      <c r="C9" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>